<commit_message>
v0.6.1 - receitas dinamicas e estrutura financeira
</commit_message>
<xml_diff>
--- a/ControleFinanceiro_2026_Prototipo_v3.xlsx
+++ b/ControleFinanceiro_2026_Prototipo_v3.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1800" yWindow="1380" windowWidth="21600" windowHeight="11385" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Configuracoes" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +40,12 @@
       <sz val="11"/>
       <u val="single"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -62,10 +68,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,105 +499,146 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9.7109375" customWidth="1" min="1" max="1"/>
-    <col width="12.140625" customWidth="1" min="2" max="2"/>
-    <col width="9.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="17.85546875" customWidth="1" min="4" max="4"/>
-    <col width="10.5703125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="12.5703125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="10.7109375" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
+    <col width="9.7109375" customWidth="1" min="2" max="2"/>
+    <col width="12.140625" customWidth="1" min="3" max="3"/>
+    <col width="9.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="17.85546875" customWidth="1" min="5" max="5"/>
+    <col width="10.5703125" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="12.5703125" bestFit="1" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
+          <t>Natureza</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Meio</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Descricao</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Valor Total</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Parcelas</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor Parcela</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>12/06/26</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>pix</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>alimentacao</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>almoco</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>25.9</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>12/06/26</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>14/06/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pix</t>
+          <t>receita</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>alimentacao</t>
+          <t>salario</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>almoco</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+          <t>trabalho</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>salario junho</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>14/06/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>despesa</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>cartao de credito</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>lazer</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>netflix</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>100</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: implementa geração de resumo de faturas
</commit_message>
<xml_diff>
--- a/ControleFinanceiro_2026_Prototipo_v3.xlsx
+++ b/ControleFinanceiro_2026_Prototipo_v3.xlsx
@@ -2006,7 +2006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2033,6 +2033,346 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>222.22</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Fechada</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>10/04/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>222.22</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Fechada</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>222.22</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Fechada</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>222.22</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Fechada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>605.55</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Fechada</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>08/2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>605.55</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Aberta</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10/09/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>605.55</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Prevista</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>10/2026</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>522.22</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Prevista</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>11/2026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10/11/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>522.22</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Prevista</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>12/2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10/12/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>522.22</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Prevista</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>01/2027</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10/01/2027</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>522.22</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Prevista</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>02/2027</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>10/02/2027</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>522.22</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Prevista</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>03/2027</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10/03/2027</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>522.22</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Prevista</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10/04/2027</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>522.22</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Prevista</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>05/2027</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10/05/2027</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>522.22</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Prevista</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>06/2027</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10/06/2027</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>822.22</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Prevista</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>07/2027</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10/07/2027</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>222.22</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Prevista</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: atualiza aba Faturas automaticamente após movimentações
</commit_message>
<xml_diff>
--- a/ControleFinanceiro_2026_Prototipo_v3.xlsx
+++ b/ControleFinanceiro_2026_Prototipo_v3.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.7109375" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -745,7 +745,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04/07/2026</t>
+          <t>03/07/2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>refil barbeador (1/1)</t>
+          <t>refil (1/1)</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -835,7 +835,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>24/08/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -850,22 +850,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>teste</t>
+          <t>alimentaçao</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>exclusao (2/3)</t>
+          <t>mercado (3/3)</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>40</v>
+        <v>74.59999999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -880,45 +880,15 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>alimentaçao</t>
+          <t>teste</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>mercado (3/3)</t>
+          <t>exclusao (3/3)</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>74.59999999999999</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>24/09/2026</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>despesa</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>credito</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>teste</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>exclusao (3/3)</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
         <v>40</v>
       </c>
     </row>
@@ -989,7 +959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1031,7 +1001,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>121.09</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1051,7 +1021,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>188.54</v>
+        <v>235.03</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1071,9 +1041,29 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>74.59999999999999</v>
+        <v>114.6</v>
       </c>
       <c r="D4" t="inlineStr">
+        <is>
+          <t>Prevista</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>10/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>40</v>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>Prevista</t>
         </is>

</xml_diff>

<commit_message>
docs: atualiza README e conclui migração para Excel
</commit_message>
<xml_diff>
--- a/ControleFinanceiro_2026_Prototipo_v3.xlsx
+++ b/ControleFinanceiro_2026_Prototipo_v3.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.7109375" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -745,7 +745,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03/07/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -760,22 +760,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>higiene</t>
+          <t>alimentaçao</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>refil (1/1)</t>
+          <t>mercado (1/1)</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>22</v>
+        <v>91.94</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>mercado (1/1)</t>
+          <t>mercado (2/3)</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>91.94</v>
+        <v>74.59999999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>28/08/2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>mercado (2/3)</t>
+          <t>mercado (3/3)</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -835,7 +835,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>28/08/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -850,45 +850,15 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>alimentaçao</t>
+          <t>teste</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>mercado (3/3)</t>
+          <t>exclusao (3/3)</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>74.59999999999999</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>24/09/2026</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>despesa</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>credito</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>teste</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>exclusao (3/3)</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1021,7 +991,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>235.03</v>
+        <v>213.03</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1041,7 +1011,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>114.6</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: conclui planejamento da interface gráfica (v0.9)
</commit_message>
<xml_diff>
--- a/ControleFinanceiro_2026_Prototipo_v3.xlsx
+++ b/ControleFinanceiro_2026_Prototipo_v3.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="EstaPastaDeTrabalho"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Configuracoes" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,6 +11,7 @@
     <sheet name="CompromissosMensais" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Faturas" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Categorias" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +41,14 @@
       <family val="2"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -62,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -70,6 +79,15 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1050,157 +1068,419 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>DASHBOARD FINANCEIRO</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Mes Selecionado:</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Ano Selecionado:</t>
-        </is>
-      </c>
+      <c r="A1" s="1" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>PLANEJAMENTO</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Receita Mensal</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Valor a Guardar</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Gastos Fixos</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Orcamento Disponivel</t>
-        </is>
-      </c>
+      <c r="A4" s="1" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>GASTOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>PIX</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Debito</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Dinheiro</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Cartao</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Total Gasto</t>
-        </is>
-      </c>
+      <c r="A11" s="1" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>INDICADOR PRINCIPAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Saldo Disponivel</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Situacao</t>
-        </is>
-      </c>
+      <c r="A19" s="1" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>FATURA</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Fatura Atual</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Proxima Fatura</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Comprometimento Futuro</t>
-        </is>
-      </c>
+      <c r="A25" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18.7109375" customWidth="1" min="1" max="1"/>
+    <col width="18.5703125" customWidth="1" min="2" max="2"/>
+    <col width="19.42578125" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Natureza</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Ativa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Freelancer</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Investimentos</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Investimentos</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Reembolso</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Venda</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Outras Receitas</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Alimentação</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Mercado</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Moradia</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Saúde</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Educação</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Lazer</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Equipamentos</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Impostos</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Assinaturas</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Vestuário</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Presentes</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Despesa</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: ajusta leitura de receitas e calculos atuais
</commit_message>
<xml_diff>
--- a/ControleFinanceiro_2026_Prototipo_v3.xlsx
+++ b/ControleFinanceiro_2026_Prototipo_v3.xlsx
@@ -8,23 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mateus\PROJETOS\meu_controle-financeiro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C66847F-99A3-4179-99F5-2D8FF46D27E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F204E47A-7F74-4C6F-B22F-D33A881CD625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuracoes" sheetId="1" r:id="rId1"/>
     <sheet name="Movimentacoes" sheetId="2" r:id="rId2"/>
     <sheet name="CompromissosMensais" sheetId="3" r:id="rId3"/>
     <sheet name="Faturas" sheetId="4" r:id="rId4"/>
-    <sheet name="Categorias" sheetId="6" r:id="rId5"/>
+    <sheet name="Categorias" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="167">
   <si>
     <t>Campo</t>
   </si>
@@ -65,85 +65,259 @@
     <t>Valor Total</t>
   </si>
   <si>
-    <t>Parcelas</t>
+    <t>23/03/2026</t>
+  </si>
+  <si>
+    <t>despesa</t>
+  </si>
+  <si>
+    <t>credito</t>
+  </si>
+  <si>
+    <t>Equipamentos</t>
+  </si>
+  <si>
+    <t>celular (1/18)</t>
+  </si>
+  <si>
+    <t>1/18</t>
+  </si>
+  <si>
+    <t>23/04/2026</t>
+  </si>
+  <si>
+    <t>celular (2/18)</t>
+  </si>
+  <si>
+    <t>2/18</t>
+  </si>
+  <si>
+    <t>23/05/2026</t>
+  </si>
+  <si>
+    <t>celular (3/18)</t>
+  </si>
+  <si>
+    <t>3/18</t>
+  </si>
+  <si>
+    <t>23/06/2026</t>
+  </si>
+  <si>
+    <t>celular (4/18)</t>
+  </si>
+  <si>
+    <t>4/18</t>
+  </si>
+  <si>
+    <t>27/06/2026</t>
+  </si>
+  <si>
+    <t>Presente</t>
+  </si>
+  <si>
+    <t>tenis olivia (1/2)</t>
+  </si>
+  <si>
+    <t>1/2</t>
   </si>
   <si>
     <t>28/06/2026</t>
   </si>
   <si>
-    <t>despesa</t>
-  </si>
-  <si>
-    <t>credito</t>
-  </si>
-  <si>
-    <t>alimentaçao</t>
-  </si>
-  <si>
-    <t>mercado (1/3)</t>
+    <t>Alimentação</t>
+  </si>
+  <si>
+    <t>sup bh (1/3)</t>
+  </si>
+  <si>
+    <t>1/3</t>
+  </si>
+  <si>
+    <t>Mercado</t>
+  </si>
+  <si>
+    <t>superminas (1/3)</t>
+  </si>
+  <si>
+    <t>06/07/2026</t>
+  </si>
+  <si>
+    <t>ASsinaturas</t>
+  </si>
+  <si>
+    <t>spotfy (1/1)</t>
+  </si>
+  <si>
+    <t>1/1</t>
+  </si>
+  <si>
+    <t>23/07/2026</t>
+  </si>
+  <si>
+    <t>celular (5/18)</t>
+  </si>
+  <si>
+    <t>5/18</t>
+  </si>
+  <si>
+    <t>27/07/2026</t>
+  </si>
+  <si>
+    <t>tenis olivia (2/2)</t>
+  </si>
+  <si>
+    <t>2/2</t>
+  </si>
+  <si>
+    <t>28/07/2026</t>
+  </si>
+  <si>
+    <t>sup bh (2/3)</t>
+  </si>
+  <si>
+    <t>2/3</t>
+  </si>
+  <si>
+    <t>superminas (2/3)</t>
+  </si>
+  <si>
+    <t>Receita</t>
   </si>
   <si>
     <t>dinheiro</t>
   </si>
   <si>
-    <t>pet</t>
-  </si>
-  <si>
-    <t>raçao doo gato</t>
-  </si>
-  <si>
-    <t>29/06/2026</t>
-  </si>
-  <si>
-    <t>pix</t>
-  </si>
-  <si>
-    <t>salgodo</t>
-  </si>
-  <si>
-    <t>02/07/2026</t>
-  </si>
-  <si>
-    <t>pao</t>
-  </si>
-  <si>
-    <t>03/07/2026</t>
-  </si>
-  <si>
-    <t>receita</t>
-  </si>
-  <si>
-    <t>salario</t>
-  </si>
-  <si>
-    <t>ifood (1/1)</t>
-  </si>
-  <si>
-    <t>06/07/2026</t>
-  </si>
-  <si>
-    <t>mercado (1/1)</t>
-  </si>
-  <si>
-    <t>28/07/2026</t>
-  </si>
-  <si>
-    <t>mercado (2/3)</t>
+    <t>Salario</t>
+  </si>
+  <si>
+    <t>23/08/2026</t>
+  </si>
+  <si>
+    <t>celular (6/18)</t>
+  </si>
+  <si>
+    <t>6/18</t>
   </si>
   <si>
     <t>28/08/2026</t>
   </si>
   <si>
-    <t>mercado (3/3)</t>
-  </si>
-  <si>
-    <t>24/09/2026</t>
-  </si>
-  <si>
-    <t>teste</t>
-  </si>
-  <si>
-    <t>exclusao (3/3)</t>
+    <t>sup bh (3/3)</t>
+  </si>
+  <si>
+    <t>3/3</t>
+  </si>
+  <si>
+    <t>superminas (3/3)</t>
+  </si>
+  <si>
+    <t>23/09/2026</t>
+  </si>
+  <si>
+    <t>celular (7/18)</t>
+  </si>
+  <si>
+    <t>7/18</t>
+  </si>
+  <si>
+    <t>23/10/2026</t>
+  </si>
+  <si>
+    <t>celular (8/18)</t>
+  </si>
+  <si>
+    <t>8/18</t>
+  </si>
+  <si>
+    <t>23/11/2026</t>
+  </si>
+  <si>
+    <t>celular (9/18)</t>
+  </si>
+  <si>
+    <t>9/18</t>
+  </si>
+  <si>
+    <t>23/12/2026</t>
+  </si>
+  <si>
+    <t>celular (10/18)</t>
+  </si>
+  <si>
+    <t>10/18</t>
+  </si>
+  <si>
+    <t>23/01/2027</t>
+  </si>
+  <si>
+    <t>celular (11/18)</t>
+  </si>
+  <si>
+    <t>11/18</t>
+  </si>
+  <si>
+    <t>23/02/2027</t>
+  </si>
+  <si>
+    <t>celular (12/18)</t>
+  </si>
+  <si>
+    <t>12/18</t>
+  </si>
+  <si>
+    <t>23/03/2027</t>
+  </si>
+  <si>
+    <t>celular (13/18)</t>
+  </si>
+  <si>
+    <t>13/18</t>
+  </si>
+  <si>
+    <t>23/04/2027</t>
+  </si>
+  <si>
+    <t>celular (14/18)</t>
+  </si>
+  <si>
+    <t>14/18</t>
+  </si>
+  <si>
+    <t>23/05/2027</t>
+  </si>
+  <si>
+    <t>celular (15/18)</t>
+  </si>
+  <si>
+    <t>15/18</t>
+  </si>
+  <si>
+    <t>23/06/2027</t>
+  </si>
+  <si>
+    <t>celular (16/18)</t>
+  </si>
+  <si>
+    <t>16/18</t>
+  </si>
+  <si>
+    <t>23/07/2027</t>
+  </si>
+  <si>
+    <t>celular (17/18)</t>
+  </si>
+  <si>
+    <t>17/18</t>
+  </si>
+  <si>
+    <t>23/08/2027</t>
+  </si>
+  <si>
+    <t>celular (18/18)</t>
+  </si>
+  <si>
+    <t>18/18</t>
   </si>
   <si>
     <t>vivo</t>
@@ -167,37 +341,121 @@
     <t>Status</t>
   </si>
   <si>
+    <t>04/2026</t>
+  </si>
+  <si>
+    <t>10/04/2026</t>
+  </si>
+  <si>
+    <t>Fechada</t>
+  </si>
+  <si>
+    <t>05/2026</t>
+  </si>
+  <si>
+    <t>10/05/2026</t>
+  </si>
+  <si>
+    <t>06/2026</t>
+  </si>
+  <si>
+    <t>10/06/2026</t>
+  </si>
+  <si>
     <t>07/2026</t>
   </si>
   <si>
     <t>10/07/2026</t>
   </si>
   <si>
-    <t>Fechada</t>
-  </si>
-  <si>
     <t>08/2026</t>
   </si>
   <si>
     <t>10/08/2026</t>
   </si>
   <si>
+    <t>09/2026</t>
+  </si>
+  <si>
+    <t>10/09/2026</t>
+  </si>
+  <si>
     <t>Aberta</t>
   </si>
   <si>
-    <t>09/2026</t>
-  </si>
-  <si>
-    <t>10/09/2026</t>
+    <t>10/2026</t>
+  </si>
+  <si>
+    <t>10/10/2026</t>
   </si>
   <si>
     <t>Prevista</t>
   </si>
   <si>
-    <t>10/2026</t>
-  </si>
-  <si>
-    <t>10/10/2026</t>
+    <t>11/2026</t>
+  </si>
+  <si>
+    <t>10/11/2026</t>
+  </si>
+  <si>
+    <t>12/2026</t>
+  </si>
+  <si>
+    <t>10/12/2026</t>
+  </si>
+  <si>
+    <t>01/2027</t>
+  </si>
+  <si>
+    <t>10/01/2027</t>
+  </si>
+  <si>
+    <t>02/2027</t>
+  </si>
+  <si>
+    <t>10/02/2027</t>
+  </si>
+  <si>
+    <t>03/2027</t>
+  </si>
+  <si>
+    <t>10/03/2027</t>
+  </si>
+  <si>
+    <t>04/2027</t>
+  </si>
+  <si>
+    <t>10/04/2027</t>
+  </si>
+  <si>
+    <t>05/2027</t>
+  </si>
+  <si>
+    <t>10/05/2027</t>
+  </si>
+  <si>
+    <t>06/2027</t>
+  </si>
+  <si>
+    <t>10/06/2027</t>
+  </si>
+  <si>
+    <t>07/2027</t>
+  </si>
+  <si>
+    <t>10/07/2027</t>
+  </si>
+  <si>
+    <t>08/2027</t>
+  </si>
+  <si>
+    <t>10/08/2027</t>
+  </si>
+  <si>
+    <t>09/2027</t>
+  </si>
+  <si>
+    <t>10/09/2027</t>
   </si>
   <si>
     <t>Nome</t>
@@ -209,13 +467,10 @@
     <t>Salário</t>
   </si>
   <si>
-    <t>Receita</t>
-  </si>
-  <si>
     <t>Sim</t>
   </si>
   <si>
-    <t>Freelancer</t>
+    <t>renda extra</t>
   </si>
   <si>
     <t>Investimentos</t>
@@ -233,12 +488,6 @@
     <t>Outras Receitas</t>
   </si>
   <si>
-    <t>Alimentação</t>
-  </si>
-  <si>
-    <t>Mercado</t>
-  </si>
-  <si>
     <t>Moradia</t>
   </si>
   <si>
@@ -257,9 +506,6 @@
     <t>Pets</t>
   </si>
   <si>
-    <t>Equipamentos</t>
-  </si>
-  <si>
     <t>Impostos</t>
   </si>
   <si>
@@ -273,6 +519,12 @@
   </si>
   <si>
     <t>Outros</t>
+  </si>
+  <si>
+    <t>emprestimo</t>
+  </si>
+  <si>
+    <t>sim</t>
   </si>
 </sst>
 </file>
@@ -709,13 +961,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Planilha2"/>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" style="4" customWidth="1"/>
     <col min="2" max="2" width="9.7109375" customWidth="1"/>
     <col min="3" max="3" width="12.140625" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" style="6" bestFit="1" customWidth="1"/>
   </cols>
@@ -739,48 +991,52 @@
       <c r="F1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
         <v>16</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2">
+        <v>263.68</v>
+      </c>
+      <c r="G2" t="s">
         <v>18</v>
-      </c>
-      <c r="F2">
-        <v>74.599999999999994</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3">
+        <v>263.68</v>
+      </c>
+      <c r="G3" t="s">
         <v>21</v>
-      </c>
-      <c r="F3">
-        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -788,19 +1044,22 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
         <v>23</v>
       </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="F4">
+        <v>263.68</v>
+      </c>
+      <c r="G4" t="s">
         <v>24</v>
-      </c>
-      <c r="F4">
-        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -808,139 +1067,571 @@
         <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
         <v>26</v>
       </c>
       <c r="F5">
-        <v>16.71</v>
+        <v>263.68</v>
+      </c>
+      <c r="G5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
         <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F6">
-        <v>2000</v>
+        <v>56.4</v>
+      </c>
+      <c r="G6" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F7">
-        <v>46.49</v>
+        <v>65.09</v>
+      </c>
+      <c r="G7" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="F8">
-        <v>91.94</v>
+        <v>74.599999999999994</v>
+      </c>
+      <c r="G8" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="F9">
-        <v>74.599999999999994</v>
+        <v>12.9</v>
+      </c>
+      <c r="G9" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s">
         <v>16</v>
       </c>
-      <c r="D10" t="s">
-        <v>17</v>
-      </c>
       <c r="E10" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="F10">
-        <v>74.599999999999994</v>
+        <v>263.68</v>
+      </c>
+      <c r="G10" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11">
+        <v>56.4</v>
+      </c>
+      <c r="G11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12">
+        <v>65.09</v>
+      </c>
+      <c r="G12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F13">
+        <v>74.599999999999994</v>
+      </c>
+      <c r="G13" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>46237</v>
+      </c>
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" t="s">
         <v>16</v>
       </c>
-      <c r="D11" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F11">
-        <v>40</v>
+      <c r="E15" t="s">
+        <v>56</v>
+      </c>
+      <c r="F15">
+        <v>263.68</v>
+      </c>
+      <c r="G15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" t="s">
+        <v>59</v>
+      </c>
+      <c r="F16">
+        <v>65.09</v>
+      </c>
+      <c r="G16" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" t="s">
+        <v>61</v>
+      </c>
+      <c r="F17">
+        <v>74.599999999999994</v>
+      </c>
+      <c r="G17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" t="s">
+        <v>63</v>
+      </c>
+      <c r="F18">
+        <v>263.68</v>
+      </c>
+      <c r="G18" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" t="s">
+        <v>66</v>
+      </c>
+      <c r="F19">
+        <v>263.68</v>
+      </c>
+      <c r="G19" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" t="s">
+        <v>69</v>
+      </c>
+      <c r="F20">
+        <v>263.68</v>
+      </c>
+      <c r="G20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>71</v>
+      </c>
+      <c r="B21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" t="s">
+        <v>72</v>
+      </c>
+      <c r="F21">
+        <v>263.68</v>
+      </c>
+      <c r="G21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" t="s">
+        <v>75</v>
+      </c>
+      <c r="F22">
+        <v>263.68</v>
+      </c>
+      <c r="G22" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>77</v>
+      </c>
+      <c r="B23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" t="s">
+        <v>78</v>
+      </c>
+      <c r="F23">
+        <v>263.68</v>
+      </c>
+      <c r="G23" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" t="s">
+        <v>16</v>
+      </c>
+      <c r="E24" t="s">
+        <v>81</v>
+      </c>
+      <c r="F24">
+        <v>263.68</v>
+      </c>
+      <c r="G24" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>83</v>
+      </c>
+      <c r="B25" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" t="s">
+        <v>16</v>
+      </c>
+      <c r="E25" t="s">
+        <v>84</v>
+      </c>
+      <c r="F25">
+        <v>263.68</v>
+      </c>
+      <c r="G25" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>86</v>
+      </c>
+      <c r="B26" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" t="s">
+        <v>16</v>
+      </c>
+      <c r="E26" t="s">
+        <v>87</v>
+      </c>
+      <c r="F26">
+        <v>263.68</v>
+      </c>
+      <c r="G26" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>89</v>
+      </c>
+      <c r="B27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" t="s">
+        <v>16</v>
+      </c>
+      <c r="E27" t="s">
+        <v>90</v>
+      </c>
+      <c r="F27">
+        <v>263.68</v>
+      </c>
+      <c r="G27" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>92</v>
+      </c>
+      <c r="B28" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" t="s">
+        <v>16</v>
+      </c>
+      <c r="E28" t="s">
+        <v>93</v>
+      </c>
+      <c r="F28">
+        <v>263.68</v>
+      </c>
+      <c r="G28" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>95</v>
+      </c>
+      <c r="B29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29" t="s">
+        <v>96</v>
+      </c>
+      <c r="F29">
+        <v>263.68</v>
+      </c>
+      <c r="G29" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -964,7 +1655,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>98</v>
       </c>
       <c r="B2">
         <v>69</v>
@@ -972,7 +1663,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>99</v>
       </c>
       <c r="B3">
         <v>642.26</v>
@@ -980,7 +1671,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>100</v>
       </c>
       <c r="B4">
         <v>12.9</v>
@@ -994,7 +1685,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Planilha4"/>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
@@ -1004,72 +1695,268 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>102</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>45</v>
+        <v>103</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>46</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>105</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>106</v>
       </c>
       <c r="C2">
-        <v>74.599999999999994</v>
+        <v>263.68</v>
       </c>
       <c r="D2" t="s">
-        <v>49</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>108</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>109</v>
       </c>
       <c r="C3">
-        <v>213.03</v>
+        <v>263.68</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>110</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="C4">
-        <v>74.599999999999994</v>
+        <v>263.68</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>112</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>113</v>
       </c>
       <c r="C5">
-        <v>40</v>
+        <v>459.77</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C6">
+        <v>472.67</v>
+      </c>
+      <c r="D6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7">
+        <v>403.37</v>
+      </c>
+      <c r="D7" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8">
+        <v>263.68</v>
+      </c>
+      <c r="D8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B9" t="s">
+        <v>123</v>
+      </c>
+      <c r="C9">
+        <v>263.68</v>
+      </c>
+      <c r="D9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>124</v>
+      </c>
+      <c r="B10" t="s">
+        <v>125</v>
+      </c>
+      <c r="C10">
+        <v>263.68</v>
+      </c>
+      <c r="D10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B11" t="s">
+        <v>127</v>
+      </c>
+      <c r="C11">
+        <v>263.68</v>
+      </c>
+      <c r="D11" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" t="s">
+        <v>129</v>
+      </c>
+      <c r="C12">
+        <v>263.68</v>
+      </c>
+      <c r="D12" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>130</v>
+      </c>
+      <c r="B13" t="s">
+        <v>131</v>
+      </c>
+      <c r="C13">
+        <v>263.68</v>
+      </c>
+      <c r="D13" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B14" t="s">
+        <v>133</v>
+      </c>
+      <c r="C14">
+        <v>263.68</v>
+      </c>
+      <c r="D14" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>134</v>
+      </c>
+      <c r="B15" t="s">
+        <v>135</v>
+      </c>
+      <c r="C15">
+        <v>263.68</v>
+      </c>
+      <c r="D15" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>136</v>
+      </c>
+      <c r="B16" t="s">
+        <v>137</v>
+      </c>
+      <c r="C16">
+        <v>263.68</v>
+      </c>
+      <c r="D16" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>138</v>
+      </c>
+      <c r="B17" t="s">
+        <v>139</v>
+      </c>
+      <c r="C17">
+        <v>263.68</v>
+      </c>
+      <c r="D17" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>140</v>
+      </c>
+      <c r="B18" t="s">
+        <v>141</v>
+      </c>
+      <c r="C18">
+        <v>263.68</v>
+      </c>
+      <c r="D18" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>142</v>
+      </c>
+      <c r="B19" t="s">
+        <v>143</v>
+      </c>
+      <c r="C19">
+        <v>263.68</v>
+      </c>
+      <c r="D19" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -1078,8 +1965,8 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:C22"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -1089,244 +1976,255 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>58</v>
+        <v>144</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>8</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>59</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>60</v>
+        <v>146</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>63</v>
+        <v>148</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>64</v>
+        <v>149</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>64</v>
+        <v>149</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>66</v>
+        <v>151</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>67</v>
+        <v>152</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>68</v>
+        <v>153</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>71</v>
+        <v>154</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>73</v>
+        <v>156</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>74</v>
+        <v>157</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>75</v>
+        <v>158</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>76</v>
+        <v>159</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>77</v>
+        <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>78</v>
+        <v>160</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>79</v>
+        <v>161</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>80</v>
+        <v>162</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>81</v>
+        <v>163</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>82</v>
+        <v>164</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>62</v>
+        <v>147</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: adiciona antecipacao de parcelas e ajustes financeiros
</commit_message>
<xml_diff>
--- a/ControleFinanceiro_2026_Prototipo_v3.xlsx
+++ b/ControleFinanceiro_2026_Prototipo_v3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mateus\PROJETOS\meu_controle-financeiro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F204E47A-7F74-4C6F-B22F-D33A881CD625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A3CDC77-1922-4613-9A0E-BED2096DF5F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11385" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuracoes" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="177">
   <si>
     <t>Campo</t>
   </si>
@@ -320,6 +320,42 @@
     <t>18/18</t>
   </si>
   <si>
+    <t>10/08/2026</t>
+  </si>
+  <si>
+    <t>pix</t>
+  </si>
+  <si>
+    <t>impostos</t>
+  </si>
+  <si>
+    <t>iptu nova uniao</t>
+  </si>
+  <si>
+    <t>06/08/2026</t>
+  </si>
+  <si>
+    <t>assinatura</t>
+  </si>
+  <si>
+    <t>receita</t>
+  </si>
+  <si>
+    <t>outras receitas</t>
+  </si>
+  <si>
+    <t>ja existia antes de começar os lançamentos</t>
+  </si>
+  <si>
+    <t>11/08/2026</t>
+  </si>
+  <si>
+    <t>renda extra</t>
+  </si>
+  <si>
+    <t>concerto celular dalina</t>
+  </si>
+  <si>
     <t>vivo</t>
   </si>
   <si>
@@ -371,9 +407,6 @@
     <t>08/2026</t>
   </si>
   <si>
-    <t>10/08/2026</t>
-  </si>
-  <si>
     <t>09/2026</t>
   </si>
   <si>
@@ -468,9 +501,6 @@
   </si>
   <si>
     <t>Sim</t>
-  </si>
-  <si>
-    <t>renda extra</t>
   </si>
   <si>
     <t>Investimentos</t>
@@ -582,12 +612,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -595,6 +623,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -961,19 +998,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Planilha2"/>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" style="7" customWidth="1"/>
     <col min="2" max="2" width="9.7109375" customWidth="1"/>
     <col min="3" max="3" width="12.140625" customWidth="1"/>
     <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="14" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -988,13 +1025,13 @@
       <c r="E1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="9" t="s">
         <v>13</v>
       </c>
       <c r="B2" t="s">
@@ -1017,7 +1054,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B3" t="s">
@@ -1040,7 +1077,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="9" t="s">
         <v>22</v>
       </c>
       <c r="B4" t="s">
@@ -1063,7 +1100,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="9" t="s">
         <v>25</v>
       </c>
       <c r="B5" t="s">
@@ -1086,7 +1123,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="9" t="s">
         <v>28</v>
       </c>
       <c r="B6" t="s">
@@ -1109,7 +1146,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="9" t="s">
         <v>32</v>
       </c>
       <c r="B7" t="s">
@@ -1132,7 +1169,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="9" t="s">
         <v>32</v>
       </c>
       <c r="B8" t="s">
@@ -1155,7 +1192,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A9" s="9" t="s">
         <v>38</v>
       </c>
       <c r="B9" t="s">
@@ -1178,7 +1215,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="A10" s="9" t="s">
         <v>42</v>
       </c>
       <c r="B10" t="s">
@@ -1201,7 +1238,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="9" t="s">
         <v>45</v>
       </c>
       <c r="B11" t="s">
@@ -1224,7 +1261,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="A12" s="9" t="s">
         <v>48</v>
       </c>
       <c r="B12" t="s">
@@ -1247,8 +1284,8 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>48</v>
+      <c r="A13" s="7">
+        <v>46205</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
@@ -1270,7 +1307,7 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="4">
+      <c r="A14" s="7">
         <v>46237</v>
       </c>
       <c r="B14" t="s">
@@ -1290,7 +1327,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="A15" s="9" t="s">
         <v>55</v>
       </c>
       <c r="B15" t="s">
@@ -1313,7 +1350,7 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="9" t="s">
         <v>58</v>
       </c>
       <c r="B16" t="s">
@@ -1336,8 +1373,8 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>58</v>
+      <c r="A17" s="7">
+        <v>46206</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
@@ -1359,7 +1396,7 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="A18" s="9" t="s">
         <v>62</v>
       </c>
       <c r="B18" t="s">
@@ -1382,7 +1419,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="A19" s="9" t="s">
         <v>65</v>
       </c>
       <c r="B19" t="s">
@@ -1405,7 +1442,7 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="A20" s="9" t="s">
         <v>68</v>
       </c>
       <c r="B20" t="s">
@@ -1428,7 +1465,7 @@
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="A21" s="9" t="s">
         <v>71</v>
       </c>
       <c r="B21" t="s">
@@ -1451,7 +1488,7 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="A22" s="9" t="s">
         <v>74</v>
       </c>
       <c r="B22" t="s">
@@ -1474,7 +1511,7 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="A23" s="9" t="s">
         <v>77</v>
       </c>
       <c r="B23" t="s">
@@ -1497,7 +1534,7 @@
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="A24" s="9" t="s">
         <v>80</v>
       </c>
       <c r="B24" t="s">
@@ -1520,7 +1557,7 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="A25" s="9" t="s">
         <v>83</v>
       </c>
       <c r="B25" t="s">
@@ -1543,7 +1580,7 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="A26" s="9" t="s">
         <v>86</v>
       </c>
       <c r="B26" t="s">
@@ -1566,7 +1603,7 @@
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="A27" s="9" t="s">
         <v>89</v>
       </c>
       <c r="B27" t="s">
@@ -1589,7 +1626,7 @@
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="A28" s="9" t="s">
         <v>92</v>
       </c>
       <c r="B28" t="s">
@@ -1612,7 +1649,7 @@
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="A29" s="9" t="s">
         <v>95</v>
       </c>
       <c r="B29" t="s">
@@ -1632,6 +1669,89 @@
       </c>
       <c r="G29" t="s">
         <v>97</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B30" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" t="s">
+        <v>99</v>
+      </c>
+      <c r="D30" t="s">
+        <v>100</v>
+      </c>
+      <c r="E30" t="s">
+        <v>101</v>
+      </c>
+      <c r="F30">
+        <v>35.700000000000003</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>102</v>
+      </c>
+      <c r="B31" t="s">
+        <v>14</v>
+      </c>
+      <c r="C31" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" t="s">
+        <v>103</v>
+      </c>
+      <c r="E31" t="s">
+        <v>40</v>
+      </c>
+      <c r="F31">
+        <v>12.9</v>
+      </c>
+      <c r="G31" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>98</v>
+      </c>
+      <c r="B32" t="s">
+        <v>104</v>
+      </c>
+      <c r="C32" t="s">
+        <v>53</v>
+      </c>
+      <c r="D32" t="s">
+        <v>105</v>
+      </c>
+      <c r="E32" t="s">
+        <v>106</v>
+      </c>
+      <c r="F32">
+        <v>28.7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>107</v>
+      </c>
+      <c r="B33" t="s">
+        <v>104</v>
+      </c>
+      <c r="C33" t="s">
+        <v>99</v>
+      </c>
+      <c r="D33" t="s">
+        <v>108</v>
+      </c>
+      <c r="E33" t="s">
+        <v>109</v>
+      </c>
+      <c r="F33">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1655,7 +1775,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="B2">
         <v>69</v>
@@ -1663,7 +1783,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="B3">
         <v>642.26</v>
@@ -1671,10 +1791,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B4">
-        <v>12.9</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -1695,268 +1812,268 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="B2" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="C2">
         <v>263.68</v>
       </c>
       <c r="D2" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="B3" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="C3">
         <v>263.68</v>
       </c>
       <c r="D3" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="B4" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="C4">
         <v>263.68</v>
       </c>
       <c r="D4" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="B5" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="C5">
-        <v>459.77</v>
+        <v>534.37</v>
       </c>
       <c r="D5" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="B6" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="C6">
         <v>472.67</v>
       </c>
       <c r="D6" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="B7" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="C7">
-        <v>403.37</v>
+        <v>341.67</v>
       </c>
       <c r="D7" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="B8" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="C8">
         <v>263.68</v>
       </c>
       <c r="D8" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="B9" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="C9">
         <v>263.68</v>
       </c>
       <c r="D9" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="B10" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="C10">
         <v>263.68</v>
       </c>
       <c r="D10" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="B11" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="C11">
         <v>263.68</v>
       </c>
       <c r="D11" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="B12" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="C12">
         <v>263.68</v>
       </c>
       <c r="D12" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="B13" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="C13">
         <v>263.68</v>
       </c>
       <c r="D13" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>143</v>
+      </c>
+      <c r="B14" t="s">
+        <v>144</v>
+      </c>
+      <c r="C14">
+        <v>263.68</v>
+      </c>
+      <c r="D14" t="s">
         <v>132</v>
-      </c>
-      <c r="B14" t="s">
-        <v>133</v>
-      </c>
-      <c r="C14">
-        <v>263.68</v>
-      </c>
-      <c r="D14" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="B15" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="C15">
         <v>263.68</v>
       </c>
       <c r="D15" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="B16" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="C16">
         <v>263.68</v>
       </c>
       <c r="D16" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="B17" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="C17">
         <v>263.68</v>
       </c>
       <c r="D17" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="B18" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="C18">
         <v>263.68</v>
       </c>
       <c r="D18" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="B19" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="C19">
         <v>263.68</v>
       </c>
       <c r="D19" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -1975,256 +2092,256 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="B1" s="7" t="s">
+      <c r="A1" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="7" t="s">
-        <v>145</v>
+      <c r="C1" s="5" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="B2" s="8" t="s">
+      <c r="A2" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>147</v>
+      <c r="C2" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="B3" s="8" t="s">
+      <c r="A3" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>147</v>
+      <c r="C3" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="B4" s="8" t="s">
+      <c r="A4" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>147</v>
+      <c r="C4" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>147</v>
+      <c r="A5" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>147</v>
+      <c r="C6" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="B7" s="8" t="s">
+      <c r="A7" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>147</v>
+      <c r="C7" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="B8" s="8" t="s">
+      <c r="A8" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>147</v>
+      <c r="C8" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>147</v>
+      <c r="B9" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>147</v>
+      <c r="B10" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>147</v>
+      <c r="A11" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>147</v>
+      <c r="A12" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>147</v>
+      <c r="A13" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>147</v>
+      <c r="A14" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>147</v>
-      </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>147</v>
+      <c r="A16" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>147</v>
+      <c r="B17" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>147</v>
+      <c r="C18" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>147</v>
+      <c r="A19" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>147</v>
+      <c r="A20" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>147</v>
+      <c r="A21" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>147</v>
+      <c r="A22" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>166</v>
+      <c r="A23" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: finaliza base funcional da versao 0.9.5
</commit_message>
<xml_diff>
--- a/ControleFinanceiro_2026_Prototipo_v3.xlsx
+++ b/ControleFinanceiro_2026_Prototipo_v3.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="EstaPastaDeTrabalho"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11385" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11385" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Configuracoes" sheetId="1" state="visible" r:id="rId1"/>
@@ -1683,7 +1683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1701,28 +1701,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>vivo</t>
+          <t>faculdade</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>69</v>
+        <v>642.26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>faculdade</t>
+          <t>telefone vivo</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>642.26</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">spotfy </t>
-        </is>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>